<commit_message>
cambios hechos al entregable #1
</commit_message>
<xml_diff>
--- a/Tercer entregable/G1_RaSA_PlantillaDisenioETL_Final.xlsx
+++ b/Tercer entregable/G1_RaSA_PlantillaDisenioETL_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa1e3ab30827bd9b/Documentos/CJHG/MAIT/3.2. Modelado de Datos y ETL/Entregas grupales/entrega_proyecto_MIAD_modelado_datos/Tercer entregable/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabrizio.cucina\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="842" documentId="11_571EF9E1CD016C53D82E76F2652E205602E7E58B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFF929BA-DE56-48E4-BECD-A00738F8068A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48688F4A-0780-4DCC-AF99-7FB975D31392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantillaDiseñoETL" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="101">
   <si>
     <t>Campos a incluir:</t>
   </si>
@@ -440,20 +440,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6484,7 +6484,7 @@
                 <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>T3. Asignar por defecto 333 a a CantidadLimite cuand se evidencien limites cuantitativos sin valor o con valor de cero.</a:t>
+            <a:t>T4. Asignar por defecto 333 a a CantidadLimite cuand se evidencien limites cuantitativos sin valor o con valor de cero.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -6836,58 +6836,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P176"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.86328125" customWidth="1"/>
-    <col min="6" max="6" width="39.06640625" customWidth="1"/>
+    <col min="2" max="2" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.88671875" customWidth="1"/>
+    <col min="6" max="6" width="39.109375" customWidth="1"/>
     <col min="8" max="8" width="43" customWidth="1"/>
-    <col min="10" max="10" width="27.1328125" customWidth="1"/>
-    <col min="12" max="12" width="51.1328125" customWidth="1"/>
+    <col min="10" max="10" width="27.109375" customWidth="1"/>
+    <col min="12" max="12" width="51.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="36" x14ac:dyDescent="1.05">
-      <c r="B2" s="18" t="s">
+    <row r="2" spans="1:16" ht="36.6" x14ac:dyDescent="0.7">
+      <c r="B2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-    </row>
-    <row r="4" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+    </row>
+    <row r="4" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="J4" s="15" t="s">
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="J4" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
@@ -6907,7 +6907,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>30</v>
       </c>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="D8" s="3"/>
       <c r="F8" s="1"/>
@@ -6931,7 +6931,7 @@
       </c>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
         <v>0</v>
       </c>
@@ -6943,7 +6943,7 @@
       <c r="J9" s="1"/>
       <c r="L9" s="3"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
@@ -6954,7 +6954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
@@ -6965,7 +6965,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
@@ -6995,7 +6995,7 @@
       <c r="J13" s="1"/>
       <c r="L13" s="3"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>17</v>
       </c>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="L14" s="3"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="L15" s="3"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>13</v>
       </c>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="L16" s="3"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="1"/>
       <c r="D17" s="3"/>
       <c r="F17" s="1" t="s">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L17" s="3"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="7" t="s">
         <v>1</v>
       </c>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="L18" s="3"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>12</v>
       </c>
@@ -7076,7 +7076,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
       <c r="D21" s="3"/>
       <c r="H21" s="3"/>
@@ -7098,7 +7098,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D22" s="3"/>
       <c r="H22" s="5"/>
       <c r="J22" s="1"/>
@@ -7106,7 +7106,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D23" s="3"/>
       <c r="H23" s="3"/>
       <c r="J23" s="1"/>
@@ -7114,13 +7114,13 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D24" s="3"/>
       <c r="H24" s="3"/>
       <c r="J24" s="1"/>
       <c r="L24" s="5"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D25" s="3"/>
       <c r="H25" s="3"/>
       <c r="J25" s="1"/>
@@ -7128,7 +7128,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D26" s="3"/>
       <c r="H26" s="3"/>
       <c r="J26" s="1"/>
@@ -7136,7 +7136,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D27" s="3"/>
       <c r="H27" s="3"/>
       <c r="J27" s="1"/>
@@ -7144,25 +7144,25 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D28" s="3"/>
       <c r="H28" s="3"/>
       <c r="L28" s="3"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D29" s="3"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H31" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H32" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D33" s="4" t="s">
         <v>5</v>
       </c>
@@ -7170,13 +7170,13 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="34" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D34" s="5" t="s">
         <v>6</v>
       </c>
       <c r="H34" s="5"/>
     </row>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="35" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D35" s="3" t="s">
         <v>20</v>
       </c>
@@ -7184,13 +7184,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="36" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D36" s="5"/>
       <c r="H36" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="37" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D37" s="5" t="s">
         <v>7</v>
       </c>
@@ -7198,7 +7198,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="38" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D38" s="3" t="s">
         <v>82</v>
       </c>
@@ -7206,7 +7206,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="39" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D39" s="3" t="s">
         <v>83</v>
       </c>
@@ -7214,7 +7214,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D40" s="3" t="s">
         <v>15</v>
       </c>
@@ -7222,7 +7222,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="41" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D41" s="3" t="s">
         <v>14</v>
       </c>
@@ -7230,7 +7230,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="42" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D42" s="3" t="s">
         <v>16</v>
       </c>
@@ -7238,43 +7238,43 @@
         <v>29</v>
       </c>
     </row>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="43" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D43" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="44" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D44" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="45" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D45" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.45">
+    <row r="46" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D46" s="5"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
-      <c r="F49" s="15" t="s">
+      <c r="F49" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G49" s="16"/>
-      <c r="H49" s="16"/>
-      <c r="J49" s="15" t="s">
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="J49" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-    </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="K49" s="14"/>
+      <c r="L49" s="14"/>
+    </row>
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="7" t="s">
         <v>2</v>
       </c>
@@ -7294,9 +7294,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D52" s="3"/>
       <c r="F52" s="1" t="s">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="L52" s="3"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="1"/>
       <c r="D53" s="3"/>
       <c r="F53" s="1"/>
@@ -7316,7 +7316,7 @@
       <c r="J53" s="1"/>
       <c r="L53" s="3"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="7" t="s">
         <v>0</v>
       </c>
@@ -7330,7 +7330,7 @@
       </c>
       <c r="L54" s="3"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="1" t="s">
         <v>24</v>
       </c>
@@ -7341,7 +7341,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="1" t="s">
         <v>26</v>
       </c>
@@ -7352,7 +7352,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="1" t="s">
         <v>25</v>
       </c>
@@ -7372,7 +7372,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B58" s="1" t="s">
         <v>28</v>
       </c>
@@ -7382,7 +7382,7 @@
       <c r="J58" s="1"/>
       <c r="L58" s="3"/>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="1" t="s">
         <v>29</v>
       </c>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="L59" s="3"/>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B60" s="1" t="s">
         <v>27</v>
       </c>
@@ -7410,7 +7410,7 @@
       </c>
       <c r="L60" s="3"/>
     </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B61" s="1"/>
       <c r="D61" s="3"/>
       <c r="F61" s="1"/>
@@ -7418,7 +7418,7 @@
       <c r="J61" s="1"/>
       <c r="L61" s="3"/>
     </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B62" s="7" t="s">
         <v>1</v>
       </c>
@@ -7426,28 +7426,28 @@
       <c r="H62" s="3"/>
       <c r="L62" s="3"/>
     </row>
-    <row r="63" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B63" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D63" s="3"/>
       <c r="L63" s="3"/>
     </row>
-    <row r="64" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D64" s="3"/>
       <c r="L64" s="3"/>
     </row>
-    <row r="65" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D65" s="3"/>
       <c r="L65" s="3"/>
     </row>
-    <row r="66" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B66" s="1"/>
       <c r="D66" s="3"/>
       <c r="H66" s="4" t="s">
@@ -7455,24 +7455,24 @@
       </c>
       <c r="L66" s="3"/>
     </row>
-    <row r="67" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D67" s="3"/>
       <c r="H67" s="5" t="s">
         <v>6</v>
       </c>
       <c r="L67" s="3"/>
     </row>
-    <row r="68" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D68" s="3"/>
       <c r="H68" s="8" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D69" s="3"/>
       <c r="H69" s="5"/>
     </row>
-    <row r="70" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D70" s="3"/>
       <c r="H70" s="5" t="s">
         <v>7</v>
@@ -7481,7 +7481,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D71" s="3"/>
       <c r="H71" s="8" t="s">
         <v>42</v>
@@ -7490,7 +7490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D72" s="3"/>
       <c r="H72" s="8" t="s">
         <v>43</v>
@@ -7499,110 +7499,108 @@
         <v>52</v>
       </c>
     </row>
-    <row r="73" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D73" s="3"/>
       <c r="H73" s="8" t="s">
         <v>44</v>
       </c>
       <c r="L73" s="5"/>
     </row>
-    <row r="74" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D74" s="3"/>
       <c r="H74" s="8"/>
       <c r="L74" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D75" s="3"/>
       <c r="L75" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="76" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D76" s="3"/>
       <c r="L76" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="77" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:12" x14ac:dyDescent="0.3">
       <c r="L77" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="78" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:12" x14ac:dyDescent="0.3">
       <c r="L78" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="79" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D79" s="4" t="s">
         <v>5</v>
       </c>
       <c r="L79" s="3"/>
     </row>
-    <row r="80" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D80" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D81" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="82" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D82" s="5"/>
     </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D83" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="84" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D84" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="85" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D85" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="86" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D86" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="87" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D87" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="88" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D88" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="89" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D89" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="90" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D90" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="D91" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="91" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D91" s="3"/>
+    </row>
+    <row r="92" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D92" s="5"/>
     </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="95" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B95" s="12" t="s">
         <v>54</v>
       </c>
@@ -7611,15 +7609,15 @@
       <c r="F95" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="G95" s="17"/>
-      <c r="H95" s="17"/>
+      <c r="G95" s="16"/>
+      <c r="H95" s="16"/>
       <c r="J95" s="12" t="s">
         <v>73</v>
       </c>
       <c r="K95" s="12"/>
       <c r="L95" s="12"/>
     </row>
-    <row r="97" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="97" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B97" s="7" t="s">
         <v>2</v>
       </c>
@@ -7639,7 +7637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="2:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="1" t="s">
         <v>55</v>
       </c>
@@ -7653,7 +7651,7 @@
       </c>
       <c r="L98" s="3"/>
     </row>
-    <row r="99" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="99" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B99" s="1"/>
       <c r="D99" s="3"/>
       <c r="F99" s="1"/>
@@ -7661,7 +7659,7 @@
       <c r="J99" s="1"/>
       <c r="L99" s="3"/>
     </row>
-    <row r="100" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="100" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B100" s="7" t="s">
         <v>0</v>
       </c>
@@ -7675,7 +7673,7 @@
       </c>
       <c r="L100" s="3"/>
     </row>
-    <row r="101" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="101" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B101" s="1" t="s">
         <v>19</v>
       </c>
@@ -7686,14 +7684,14 @@
         <v>60</v>
       </c>
     </row>
-    <row r="102" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="102" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B102" s="1"/>
       <c r="F102" s="1" t="s">
         <v>12</v>
       </c>
       <c r="J102" s="1"/>
     </row>
-    <row r="103" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="103" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B103" s="7" t="s">
         <v>1</v>
       </c>
@@ -7711,7 +7709,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="104" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B104" s="1" t="s">
         <v>11</v>
       </c>
@@ -7725,7 +7723,7 @@
       </c>
       <c r="L104" s="3"/>
     </row>
-    <row r="105" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="105" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
         <v>22</v>
       </c>
@@ -7739,7 +7737,7 @@
       </c>
       <c r="L105" s="3"/>
     </row>
-    <row r="106" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="106" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B106" s="1" t="s">
         <v>56</v>
       </c>
@@ -7753,7 +7751,7 @@
       </c>
       <c r="L106" s="3"/>
     </row>
-    <row r="107" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="107" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B107" s="1" t="s">
         <v>57</v>
       </c>
@@ -7767,7 +7765,7 @@
       </c>
       <c r="L107" s="3"/>
     </row>
-    <row r="108" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="108" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B108" s="1" t="s">
         <v>58</v>
       </c>
@@ -7781,7 +7779,7 @@
       </c>
       <c r="L108" s="3"/>
     </row>
-    <row r="109" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="109" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
         <v>59</v>
       </c>
@@ -7795,7 +7793,7 @@
       </c>
       <c r="L109" s="3"/>
     </row>
-    <row r="110" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="110" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
         <v>60</v>
       </c>
@@ -7809,7 +7807,7 @@
       </c>
       <c r="L110" s="3"/>
     </row>
-    <row r="111" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="111" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
         <v>61</v>
       </c>
@@ -7822,7 +7820,7 @@
       </c>
       <c r="L111" s="3"/>
     </row>
-    <row r="112" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="112" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B112" s="1" t="s">
         <v>62</v>
       </c>
@@ -7833,7 +7831,7 @@
       </c>
       <c r="L112" s="3"/>
     </row>
-    <row r="113" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="113" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
         <v>63</v>
       </c>
@@ -7846,41 +7844,41 @@
       </c>
       <c r="L113" s="3"/>
     </row>
-    <row r="114" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="114" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D114" s="3"/>
       <c r="H114" s="5" t="s">
         <v>6</v>
       </c>
       <c r="L114" s="3"/>
     </row>
-    <row r="115" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="115" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D115" s="3"/>
       <c r="H115" s="11" t="s">
         <v>69</v>
       </c>
       <c r="L115" s="3"/>
     </row>
-    <row r="116" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="116" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D116" s="3"/>
       <c r="H116" s="5"/>
       <c r="L116" s="3"/>
     </row>
-    <row r="117" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="117" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D117" s="3"/>
       <c r="H117" s="5"/>
     </row>
-    <row r="118" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="118" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D118" s="3"/>
       <c r="H118" s="5"/>
     </row>
-    <row r="119" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="119" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D119" s="3"/>
       <c r="H119" s="5"/>
       <c r="L119" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="120" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H120" s="5" t="s">
         <v>7</v>
       </c>
@@ -7888,7 +7886,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="121" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H121" s="3" t="s">
         <v>32</v>
       </c>
@@ -7896,13 +7894,13 @@
         <v>72</v>
       </c>
     </row>
-    <row r="122" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="122" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H122" s="3" t="s">
         <v>11</v>
       </c>
       <c r="L122" s="5"/>
     </row>
-    <row r="123" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="123" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D123" s="4" t="s">
         <v>5</v>
       </c>
@@ -7913,7 +7911,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="124" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D124" s="5" t="s">
         <v>6</v>
       </c>
@@ -7925,7 +7923,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="125" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="125" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D125" s="3" t="s">
         <v>64</v>
       </c>
@@ -7933,44 +7931,44 @@
         <v>74</v>
       </c>
     </row>
-    <row r="126" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="126" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D126" s="5"/>
       <c r="L126" s="5"/>
     </row>
-    <row r="127" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="127" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D127" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="128" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D128" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="129" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="129" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D129" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="130" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="130" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D130" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="131" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="131" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D131" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="132" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="132" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D132" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="133" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="133" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D133" s="5"/>
     </row>
-    <row r="136" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="136" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B136" s="12" t="s">
         <v>76</v>
       </c>
@@ -7984,7 +7982,7 @@
       <c r="I136" s="12"/>
       <c r="J136" s="12"/>
     </row>
-    <row r="138" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="138" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B138" s="7" t="s">
         <v>2</v>
       </c>
@@ -7994,13 +7992,13 @@
       <c r="F138" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="H138" s="14" t="s">
+      <c r="H138" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="I138" s="14"/>
-      <c r="J138" s="14"/>
-    </row>
-    <row r="139" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="I138" s="18"/>
+      <c r="J138" s="18"/>
+    </row>
+    <row r="139" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B139" s="1" t="s">
         <v>77</v>
       </c>
@@ -8012,7 +8010,7 @@
       <c r="I139" s="3"/>
       <c r="J139" s="3"/>
     </row>
-    <row r="140" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="140" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B140" s="1" t="s">
         <v>78</v>
       </c>
@@ -8024,7 +8022,7 @@
       <c r="I140" s="3"/>
       <c r="J140" s="3"/>
     </row>
-    <row r="141" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="141" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B141" s="1" t="s">
         <v>64</v>
       </c>
@@ -8036,7 +8034,7 @@
       <c r="I141" s="3"/>
       <c r="J141" s="3"/>
     </row>
-    <row r="142" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="142" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B142" s="1"/>
       <c r="D142" s="3"/>
       <c r="F142" s="1" t="s">
@@ -8046,7 +8044,7 @@
       <c r="I142" s="3"/>
       <c r="J142" s="3"/>
     </row>
-    <row r="143" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="143" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B143" s="7" t="s">
         <v>0</v>
       </c>
@@ -8054,7 +8052,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="144" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="144" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B144" s="1" t="s">
         <v>32</v>
       </c>
@@ -8062,7 +8060,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="145" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="145" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B145" s="1" t="s">
         <v>79</v>
       </c>
@@ -8072,13 +8070,13 @@
       <c r="F145" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="H145" s="14" t="s">
+      <c r="H145" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="I145" s="14"/>
-      <c r="J145" s="14"/>
-    </row>
-    <row r="146" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="I145" s="18"/>
+      <c r="J145" s="18"/>
+    </row>
+    <row r="146" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B146" s="1" t="s">
         <v>80</v>
       </c>
@@ -8088,7 +8086,7 @@
       <c r="I146" s="3"/>
       <c r="J146" s="3"/>
     </row>
-    <row r="147" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="147" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B147" s="1" t="s">
         <v>81</v>
       </c>
@@ -8100,7 +8098,7 @@
       <c r="I147" s="3"/>
       <c r="J147" s="3"/>
     </row>
-    <row r="148" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="148" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B148" s="1"/>
       <c r="D148" s="3"/>
       <c r="F148" s="1" t="s">
@@ -8110,7 +8108,7 @@
       <c r="I148" s="3"/>
       <c r="J148" s="3"/>
     </row>
-    <row r="149" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="149" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B149" s="7" t="s">
         <v>1</v>
       </c>
@@ -8122,7 +8120,7 @@
       <c r="I149" s="3"/>
       <c r="J149" s="3"/>
     </row>
-    <row r="150" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="150" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B150" s="1" t="s">
         <v>11</v>
       </c>
@@ -8134,7 +8132,7 @@
       <c r="I150" s="4"/>
       <c r="J150" s="4"/>
     </row>
-    <row r="151" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="151" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B151" s="1" t="s">
         <v>12</v>
       </c>
@@ -8146,7 +8144,7 @@
       <c r="I151" s="3"/>
       <c r="J151" s="3"/>
     </row>
-    <row r="152" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="152" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B152" s="1" t="s">
         <v>11</v>
       </c>
@@ -8158,7 +8156,7 @@
       <c r="I152" s="3"/>
       <c r="J152" s="3"/>
     </row>
-    <row r="153" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="153" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B153" s="1" t="s">
         <v>15</v>
       </c>
@@ -8170,7 +8168,7 @@
       <c r="I153" s="3"/>
       <c r="J153" s="3"/>
     </row>
-    <row r="154" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="154" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B154" s="1" t="s">
         <v>14</v>
       </c>
@@ -8182,7 +8180,7 @@
       <c r="I154" s="3"/>
       <c r="J154" s="3"/>
     </row>
-    <row r="155" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="155" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B155" s="1" t="s">
         <v>16</v>
       </c>
@@ -8194,7 +8192,7 @@
       <c r="I155" s="4"/>
       <c r="J155" s="4"/>
     </row>
-    <row r="156" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="156" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B156" s="1" t="s">
         <v>17</v>
       </c>
@@ -8205,7 +8203,7 @@
       <c r="I156" s="3"/>
       <c r="J156" s="3"/>
     </row>
-    <row r="157" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="157" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B157" s="1" t="s">
         <v>18</v>
       </c>
@@ -8213,7 +8211,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="158" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="158" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B158" s="1" t="s">
         <v>13</v>
       </c>
@@ -8221,7 +8219,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="159" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="159" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B159" s="1" t="s">
         <v>19</v>
       </c>
@@ -8231,13 +8229,13 @@
       <c r="F159" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H159" s="14" t="s">
+      <c r="H159" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="I159" s="14"/>
-      <c r="J159" s="14"/>
-    </row>
-    <row r="160" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="I159" s="18"/>
+      <c r="J159" s="18"/>
+    </row>
+    <row r="160" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B160" s="1" t="s">
         <v>66</v>
       </c>
@@ -8251,7 +8249,7 @@
       <c r="I160" s="3"/>
       <c r="J160" s="3"/>
     </row>
-    <row r="161" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="161" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B161" s="1" t="s">
         <v>67</v>
       </c>
@@ -8267,42 +8265,42 @@
       <c r="I161" s="3"/>
       <c r="J161" s="3"/>
     </row>
-    <row r="162" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="162" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B162" s="1" t="s">
         <v>68</v>
       </c>
       <c r="D162" s="5"/>
-      <c r="F162" s="13" t="s">
+      <c r="F162" s="17" t="s">
         <v>99</v>
       </c>
       <c r="H162" s="5"/>
       <c r="I162" s="3"/>
       <c r="J162" s="3"/>
     </row>
-    <row r="163" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="163" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B163" s="1"/>
       <c r="D163" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F163" s="13"/>
+      <c r="F163" s="17"/>
       <c r="H163" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I163" s="3"/>
       <c r="J163" s="3"/>
     </row>
-    <row r="164" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="164" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D164" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F164" s="13"/>
+      <c r="F164" s="17"/>
       <c r="H164" s="3" t="s">
         <v>88</v>
       </c>
       <c r="I164" s="4"/>
       <c r="J164" s="4"/>
     </row>
-    <row r="165" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="165" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D165" s="3" t="s">
         <v>79</v>
       </c>
@@ -8312,7 +8310,7 @@
       <c r="I165" s="3"/>
       <c r="J165" s="3"/>
     </row>
-    <row r="166" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="166" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D166" s="3" t="s">
         <v>80</v>
       </c>
@@ -8322,7 +8320,7 @@
       <c r="I166" s="3"/>
       <c r="J166" s="3"/>
     </row>
-    <row r="167" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="167" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D167" s="3" t="s">
         <v>81</v>
       </c>
@@ -8332,7 +8330,7 @@
       <c r="I167" s="3"/>
       <c r="J167" s="3"/>
     </row>
-    <row r="168" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="168" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D168" s="3" t="s">
         <v>85</v>
       </c>
@@ -8342,7 +8340,7 @@
       <c r="I168" s="3"/>
       <c r="J168" s="3"/>
     </row>
-    <row r="169" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="169" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D169" s="5"/>
       <c r="H169" s="3" t="s">
         <v>92</v>
@@ -8350,62 +8348,55 @@
       <c r="I169" s="4"/>
       <c r="J169" s="4"/>
     </row>
-    <row r="170" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="170" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H170" s="3" t="s">
         <v>93</v>
       </c>
       <c r="I170" s="4"/>
       <c r="J170" s="4"/>
     </row>
-    <row r="171" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="171" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H171" s="3" t="s">
         <v>94</v>
       </c>
       <c r="I171" s="4"/>
       <c r="J171" s="4"/>
     </row>
-    <row r="172" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="172" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H172" s="3" t="s">
         <v>95</v>
       </c>
       <c r="I172" s="4"/>
       <c r="J172" s="4"/>
     </row>
-    <row r="173" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="173" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H173" s="3" t="s">
         <v>96</v>
       </c>
       <c r="I173" s="4"/>
       <c r="J173" s="4"/>
     </row>
-    <row r="174" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="174" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H174" s="3" t="s">
         <v>97</v>
       </c>
       <c r="I174" s="4"/>
       <c r="J174" s="4"/>
     </row>
-    <row r="175" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="175" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H175" s="3" t="s">
         <v>98</v>
       </c>
       <c r="I175" s="4"/>
       <c r="J175" s="4"/>
     </row>
-    <row r="176" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="176" spans="2:10" x14ac:dyDescent="0.3">
       <c r="H176" s="5"/>
       <c r="I176" s="3"/>
       <c r="J176" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="J49:L49"/>
     <mergeCell ref="B95:D95"/>
     <mergeCell ref="F95:H95"/>
     <mergeCell ref="J95:L95"/>
@@ -8415,9 +8406,22 @@
     <mergeCell ref="F136:J136"/>
     <mergeCell ref="H145:J145"/>
     <mergeCell ref="H159:J159"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="J49:L49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{86e23165-d923-4ef0-ae5f-fd5f4d5ec307}" enabled="1" method="Standard" siteId="{eeb14196-63dc-45aa-ac42-0a4583b12590}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>